<commit_message>
Team Schedule Capture as of 10/24/2026 5:30 AM
</commit_message>
<xml_diff>
--- a/data/2026/cjsl/fall/albion-sc-brooklyn-b15-16-premier-williamsburg.xlsx
+++ b/data/2026/cjsl/fall/albion-sc-brooklyn-b15-16-premier-williamsburg.xlsx
@@ -284,7 +284,7 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0 - 2</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
@@ -304,7 +304,7 @@
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Forfeit</t>
         </is>
       </c>
     </row>

</xml_diff>